<commit_message>
Add hot-topic pipelines (India forex video + article) & Cafre templates
- india_forex_video.py: scrape India forex tweets -> AI hot topics -> combined
  news script -> in-process batch render (full video).
- india_forex_article.py: same fetch/analysis, writes Top-N editorial English
  articles with catchy headlines to output/articles_*.
- Keys read from env / gitignored keys_local.py (no plaintext secrets in repo).
- New templates: 今日_Cafre_* (Berita Broker / Global Markets / Peringatan Penipuan
  x2), 印度外汇热点, 炫富生活 variants, 风水知识英文轻悬疑.
- tagging.py: atomic write for real_footage_cache (safe under parallel batches).
- gitignore: keys_local.py, Colab secret script, stray MPY temp mp4s, unrelated dirs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/wikigold/scripts.xlsx
+++ b/templates/wikigold/scripts.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,12 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>weekend_gold_wikigold</t>
+          <t>Why Gold Is Unpredictable in India This Week</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gold prices don't wait for Monday. Global news can impact gold anytime. Stay updated with weekend gold prices using WikiGold. Track gold. Follow Indian rupee gold prices. Stay one step ahead. Download WikiGold today.</t>
+          <t>Why is gold becoming so unpredictable in India this week?
+Gold prices are facing pressure as demand slows and buyers remain cautious after recent price volatility.
+Indian jewelers are focusing more on old gold exchanges instead of fresh purchases.
+At the same time, global events, inflation concerns, and US economic policies continue to influence gold prices worldwide.
+Whether you are a gold buyer or trader, following market changes is important.
+WikiGold helps you monitor gold prices, charts, and market movements easily.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -465,12 +470,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gold_never_sleeps</t>
+          <t>Indian Gold Investors What Is Next for Gold Prices</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The gold market is closed, but gold never really sleeps. Wars. Breaking news. Central banks. Global events. By Monday, the price could already be moving. WikiGold lets you check gold prices even on weekends. Stay informed. Stay ahead. Download WikiGold today.</t>
+          <t>Indian gold investors, what's next for gold prices?
+Gold has seen strong movements this week as traders watch global markets closely.
+The US dollar, interest rate expectations, and geopolitical risks are still the biggest factors affecting gold prices.
+Many investors are asking, will gold continue rising, or is a correction coming?
+No one can predict the market perfectly, but tracking price trends and market data can help you make better decisions.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix classify_footage hang (timeout+retry) & un-ignore template configs
- tagging.py: add timeout (_CLASSIFY_TIMEOUT_MS=30s) + retry (2x) to the
  Gemini classify_footage generate_content call. Previously an unbounded
  network call could hang a render forever at the material-selection stage
  (no ffmpeg, output not growing, log stuck on classify_footage). Now it
  times out and degrades gracefully instead of blocking indefinitely.
- .gitignore: anchor secret config rule to /config.toml so it no longer
  also ignores templates/*/config.toml. Those template configs were never
  committed, so cloned templates were missing config.toml and couldn't run.
  Add all 11 template config.toml files.
- Add 今日_Cafre_Peringatan_Penipuan_C template (3-way parallel clone) and
  refresh template scripts.xlsx to latest batch content.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/wikigold/scripts.xlsx
+++ b/templates/wikigold/scripts.xlsx
@@ -446,20 +446,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Why Gold Is Unpredictable in India This Week</t>
+          <t>Gold Falls Below 4000 What Indian Investors Watch</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Why is gold becoming so unpredictable in India this week?
-Gold prices are facing pressure as demand slows and buyers remain cautious after recent price volatility.
-Indian jewelers are focusing more on old gold exchanges instead of fresh purchases.
-At the same time, global events, inflation concerns, and US economic policies continue to influence gold prices worldwide.
-Whether you are a gold buyer or trader, following market changes is important.
-WikiGold helps you monitor gold prices, charts, and market movements easily.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Gold prices have fallen below the important 4,000 dollar level.
+But surprisingly, the reason is rising Middle East tension.
+Higher oil prices are increasing inflation fears, which could push the US Federal Reserve toward higher interest rates. A stronger dollar and rising bond yields are now putting pressure on gold.
+Will gold continue falling, or is this a buying opportunity?
+Check live gold prices, market trends and important gold news anytime on the WikiGold App.
+Download WikiGold and stay ahead of the gold market.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>gold price falls below 4000 dollar Middle East tension oil inflation Fed rate dollar bond yields</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
@@ -470,19 +474,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Indian Gold Investors What Is Next for Gold Prices</t>
+          <t>Global Gold Falling But India Gold Still Expensive</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Indian gold investors, what's next for gold prices?
-Gold has seen strong movements this week as traders watch global markets closely.
-The US dollar, interest rate expectations, and geopolitical risks are still the biggest factors affecting gold prices.
-Many investors are asking, will gold continue rising, or is a correction coming?
-No one can predict the market perfectly, but tracking price trends and market data can help you make better decisions.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>International gold prices have dropped sharply, but gold in India is still trading at high levels.
+Why? Because Indian gold prices are not controlled by the global market alone.
+A weaker Indian rupee makes imported gold more expensive, while higher import duties add even more cost for Indian buyers.
+That means global gold may fall, but jewellery and investment gold prices in India may not fall by the same amount.
+Before buying gold this weekend, check the latest Indian and international gold trends on WikiGold.
+Download WikiGold for live prices, market news and gold analysis.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>India gold price high weaker rupee import duty global gold jewellery investment MCX gold rate</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>

</xml_diff>